<commit_message>
fix: hide matadata sheet in invoice
</commit_message>
<xml_diff>
--- a/xlsx/tests/templates/invoice.xlsx
+++ b/xlsx/tests/templates/invoice.xlsx
@@ -5,17 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dg-ac/Documents/IronCalc Mkt/Templates/final/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dg-ac/Documents/IronCalc Mkt/Templates/v0.8.02/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{050D83BB-4D47-A74A-8915-EC6995795A05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{334CE5B4-A02F-DD4D-AC4B-50B1D49596C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Invoice" sheetId="1" r:id="rId1"/>
     <sheet name="Settings" sheetId="2" r:id="rId2"/>
-    <sheet name="METADATA" sheetId="3" r:id="rId3"/>
+    <sheet name="METADATA" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="AccountHolder">Settings!$C$13</definedName>
@@ -958,7 +958,7 @@
       </c>
       <c r="H4" s="12">
         <f ca="1">TODAY()</f>
-        <v>46226</v>
+        <v>46233</v>
       </c>
       <c r="I4" s="2"/>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="H5" s="12">
         <f ca="1">WORKDAY(H4,PaymentTermsDays)</f>
-        <v>46268</v>
+        <v>46275</v>
       </c>
       <c r="I5" s="2"/>
     </row>
@@ -1755,7 +1755,7 @@
       </c>
       <c r="B2" s="37">
         <f ca="1">NOW()</f>
-        <v>46226.524244328706</v>
+        <v>46233.61136145833</v>
       </c>
     </row>
   </sheetData>

</xml_diff>